<commit_message>
refactor wave spawn logic
</commit_message>
<xml_diff>
--- a/images/boss_ship_64x32_packed.xlsx
+++ b/images/boss_ship_64x32_packed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/giac/Coding/cgahscroll/images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C5B3D72-E54E-C248-A313-00870BE478FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8348BCFE-D37B-3A41-8F20-1C644B35BC25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1180" windowWidth="27640" windowHeight="16640" xr2:uid="{ACEC98CD-13E3-1248-9726-5AB6616BC61F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="1">
   <si>
     <t>db</t>
   </si>
@@ -897,7 +897,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A8A109E-9D3E-2F43-B263-090D31009DB0}">
-  <dimension ref="A1:Q66"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="2:17" x14ac:dyDescent="0.2">
@@ -4706,75 +4706,6 @@
       <c r="Q65" t="str">
         <f>TEXT(VLOOKUP(Q32,Sheet1!$A$2:$L$257,12,FALSE),"0#")</f>
         <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>0</v>
-      </c>
-      <c r="B66" t="str">
-        <f>TEXT(VLOOKUP(B33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="C66" t="str">
-        <f>TEXT(VLOOKUP(C33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="D66" t="str">
-        <f>TEXT(VLOOKUP(D33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="E66" t="str">
-        <f>TEXT(VLOOKUP(E33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="F66" t="str">
-        <f>TEXT(VLOOKUP(F33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="G66" t="str">
-        <f>TEXT(VLOOKUP(G33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="H66" t="str">
-        <f>TEXT(VLOOKUP(H33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="I66" t="str">
-        <f>TEXT(VLOOKUP(I33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="J66" t="str">
-        <f>TEXT(VLOOKUP(J33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="K66" t="str">
-        <f>TEXT(VLOOKUP(K33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="L66" t="str">
-        <f>TEXT(VLOOKUP(L33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="M66" t="str">
-        <f>TEXT(VLOOKUP(M33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="N66" t="str">
-        <f>TEXT(VLOOKUP(N33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="O66" t="str">
-        <f>TEXT(VLOOKUP(O33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="P66" t="str">
-        <f>TEXT(VLOOKUP(P33,Sheet1!$A$2:$L$257,12,FALSE),"0#")&amp;","</f>
-        <v>255,</v>
-      </c>
-      <c r="Q66" t="str">
-        <f>TEXT(VLOOKUP(Q33,Sheet1!$A$2:$L$257,12,FALSE),"0#")</f>
-        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>